<commit_message>
Name the current journal throughout, and pin the two folders that are not the package
The package still carried the previous target journal's name in README.md, in the
identification banner written into every sheet of ESM_1-ESM_4, and in the
supplementary-figure source. All three now name the journal the manuscript is
submitted to; the four workbooks and Online Resource 5 are regenerated so the fix
reaches the files a reader actually opens, the digest manifest is recomputed, and
the one-file snapshot is rebuilt from the updated tree.

.gitignore additionally covers the graphical-abstract folder, the local literature
cache (the existing rule never matched that directory's name) and the working
scripts left over from the revision -- none of the three is replication material.
</commit_message>
<xml_diff>
--- a/supplementary/ESM_1.xlsx
+++ b/supplementary/ESM_1.xlsx
@@ -435,14 +435,14 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Article title: What is shared across 33 cancer types is the tissue, not the tumour: a non-malignant axis recovered only from aligned gene panels</t>
+          <t>Article title: What is shared across 33 cancer types is the tissue, not the tumour: a non-malignant axis of the microenvironment</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Journal: Functional &amp; Integrative Genomics</t>
+          <t>Journal: Network Modeling Analysis in Health Informatics and Bioinformatics</t>
         </is>
       </c>
     </row>

</xml_diff>